<commit_message>
feat(database): add AI speaking tables and payment system
- Created new enums for AI speaking session states, turn statuses, and roles.
- Added tables for ai_speaking_sessions, ai_speaking_turns, and ai_speaking_turn_segments.
- Implemented payment system with enums for payment status, provider, and transaction types.
- Altered ClassroomStudent table to include isPurchased column.
- Created Transaction table with necessary fields and foreign key constraints.
- Added ClassroomStatus enum and updated Classroom model to include status.
- Updated Prisma schema to reflect new models and enums.
- Introduced GeminiService for AI functionalities, including embedding generation and response handling.
- Added access token guard improvements for better token extraction.
- Created a script to generate test payment data for courses and classrooms.
</commit_message>
<xml_diff>
--- a/temp-uploads/family_course_import.xlsx
+++ b/temp-uploads/family_course_import.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="11200"/>
+    <workbookView windowWidth="28800" windowHeight="11260"/>
   </bookViews>
   <sheets>
     <sheet name="Courses" sheetId="1" r:id="rId1"/>
@@ -66,7 +66,7 @@
     <t>FAMILY-001</t>
   </si>
   <si>
-    <t>Gia đình - Family Course</t>
+    <t>Zoo- Sở thú cấp cao</t>
   </si>
   <si>
     <t>Khóa học tiếng Anh chủ đề Gia đình, mỗi lesson chứa đầy đủ 8 activity chuẩn để thử import.</t>
@@ -1344,6 +1344,9 @@
   <sheetPr/>
   <dimension ref="A1:K2"/>
   <sheetFormatPr defaultColWidth="7.94117647058824" defaultRowHeight="17.6" outlineLevelRow="1"/>
+  <cols>
+    <col min="4" max="4" width="12.6470588235294"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:11">
       <c r="A1" t="s">
@@ -1391,7 +1394,7 @@
         <v>13</v>
       </c>
       <c r="D2">
-        <v>200</v>
+        <v>12</v>
       </c>
       <c r="E2" t="s">
         <v>14</v>
@@ -1419,7 +1422,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
   <ignoredErrors>
-    <ignoredError sqref="A2:J2 A1:K1" numberStoredAsText="1"/>
+    <ignoredError sqref="E2:J2 C2 A2 A1:K1" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1429,6 +1432,12 @@
   <sheetPr/>
   <dimension ref="A1:AB61"/>
   <sheetFormatPr defaultColWidth="7.94117647058824" defaultRowHeight="17.6"/>
+  <cols>
+    <col min="8" max="8" width="46.8088235294118" customWidth="1"/>
+    <col min="9" max="9" width="30.0220588235294" customWidth="1"/>
+    <col min="10" max="10" width="25.4852941176471" customWidth="1"/>
+    <col min="11" max="11" width="103.426470588235" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:28">
       <c r="A1" t="s">

</xml_diff>